<commit_message>
Release warranty, gross profit, and report fixes on the existing .NET 8 and React Router 6 stack.
Keep the Verify-only import-batch migration documented and unapplied.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Documentation/samples/product-import-test.xlsx
+++ b/Documentation/samples/product-import-test.xlsx
@@ -49,6 +49,30 @@
     <x:t>OpeningStock</x:t>
   </x:si>
   <x:si>
+    <x:t>Barcode</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WarrantyValue</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WarrantyUnit</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RequiresSerial</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ProductId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>StockQuantity</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AddStockQuantity</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ReceiptId</x:t>
+  </x:si>
+  <x:si>
     <x:t>DEMO USB cable</x:t>
   </x:si>
   <x:si>
@@ -79,10 +103,10 @@
     <x:t>ProductName*  — up to 200 characters. Duplicate names are allowed.</x:t>
   </x:si>
   <x:si>
-    <x:t>SKU*          — up to 200 characters. Must be unique. Existing SKUs are skipped, never overwritten.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Category      — must match an existing category name exactly (see Lookups).</x:t>
+    <x:t>SKU*          — up to 200 characters. Unique. Matches an existing product when Product ID and barcode are blank.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Category      — must match an existing category name exactly (see Lookups). Blank on an existing product leaves the current category.</x:t>
   </x:si>
   <x:si>
     <x:t>Brand         — must match an existing brand name (see Lookups).</x:t>
@@ -94,16 +118,40 @@
     <x:t>Tax           — existing tax name (e.g. GST 18) or the rate number (e.g. 18). Inactive taxes are rejected.</x:t>
   </x:si>
   <x:si>
-    <x:t>HSN           — 4, 6 or 8 digits. Leave blank if unknown.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PurchasePrice* — rupees, 0 or more, at most 2 decimal places.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SellingPrice*  — rupees, 0 or more, at most 2 decimal places.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OpeningStock   — whole number 0 or more. Added through the stock ledger as opening stock. Leave blank for 0.</x:t>
+    <x:t>HSN           — 4, 6 or 8 digits. Leave blank if unknown. Blank does not clear an existing HSN.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PurchasePrice* — rupees, 0 or more, at most 2 decimal places. Required for new products. Blank on an existing product leaves the current price.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SellingPrice*  — rupees, 0 or more, at most 2 decimal places. Required for new products.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OpeningStock   — desired on-hand for existing products (Excel − current stock is added). Blank is NOT zero. Excel never reduces stock.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Barcode        — optional unique shop/EAN code used by POS scan. Match key #2 after Product ID.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WarrantyValue  — optional default length (whole number). Used only as a default on new sales.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WarrantyUnit   — Days, Months or Years. Required when WarrantyValue is set.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RequiresSerial — Yes or No. Serials are stored on warranty registrations, not as serial-level stock.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ProductId      — optional. Trusted match to an existing product. Do not invent IDs for new rows.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>StockQuantity  — same as OpeningStock (desired on-hand). Confirm recalculates the difference against live stock.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AddStockQuantity — Mode B: quantity to add (a delivery). Blank or 0 = no add. Do not combine with StockQuantity.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ReceiptId      — optional delivery/batch id for incremental stock. Same id cannot add twice.</x:t>
   </x:si>
   <x:si>
     <x:t>The Sample sheet is an example only and is NEVER imported.</x:t>
@@ -115,10 +163,10 @@
     <x:t>Maximum 2,000 product rows and 5 MB.</x:t>
   </x:si>
   <x:si>
-    <x:t>Retrying the same file is safe: products already imported (same SKU) are skipped, so stock is not added twice.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Existing products are never overwritten. Rows with a SKU that already exists (in the file or in the catalogue) are skipped and listed in the result. Invalid rows are reported and not imported. Valid rows are written in one transaction: they all succeed or none are saved. Opening stock goes through the stock ledger. There is no barcode or description column — those fields are not on the product. Duplicate product names are allowed; SKU must be unique. Maximum 2,000 data rows and 5 MB per file.</x:t>
+    <x:t>Retrying the same file (same bytes) returns the original result; stock is not added twice.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>A barcode or SKU that already exists is a match, not a duplicate: that product is updated. Match by barcode, then SKU (whitespace trimmed; Product ID if present). New products are added with OpeningStock as opening quantity. For existing products OpeningStock is the desired on-hand target: only (Excel − current stock) is added through the ledger. Equal quantities skip stock. Blank OpeningStock is not zero and leaves stock unchanged. Excel never reduces stock — use Inventory → Adjustments. Provided product fields are updated; blank optional cells do not clear stored values. Duplicate means the same product appears twice in this file, not that it exists in the catalogue. Confirm recalculates the difference against live stock. The same file is imported once. Applicable rows are one transaction. Maximum 2,000 rows and 5 MB.</x:t>
   </x:si>
   <x:si>
     <x:t>Categories</x:t>
@@ -166,10 +214,7 @@
     <x:t>SAMPLE-NEG-01</x:t>
   </x:si>
   <x:si>
-    <x:t>Duplicate of first</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Already in catalogue</x:t>
+    <x:t>Existing</x:t>
   </x:si>
   <x:si>
     <x:t>EXISTING-1</x:t>
@@ -558,7 +603,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:J1"/>
+  <x:dimension ref="A1:R1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14.424911" style="0" customWidth="1"/>
@@ -571,9 +616,17 @@
     <x:col min="8" max="8" width="14.567768" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="11.853482" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="8.282054" style="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14.424911" style="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13.282054" style="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="15" max="15" width="9.853482" style="0" customWidth="1"/>
+    <x:col min="16" max="16" width="13.853482" style="0" customWidth="1"/>
+    <x:col min="17" max="17" width="17.567768" style="0" customWidth="1"/>
+    <x:col min="18" max="18" width="9.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:10">
+    <x:row r="1" spans="1:18">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -604,28 +657,52 @@
       <x:c r="J1" s="1" t="s">
         <x:v>9</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:10">
+      <x:c r="K1" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L1" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="M1" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N1" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="O1" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="P1" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="Q1" s="1" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="R1" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:18">
       <x:c r="A2" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>80</x:v>
@@ -637,27 +714,27 @@
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:10">
+    <x:row r="3" spans="1:18">
       <x:c r="A3" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>150</x:v>
@@ -669,27 +746,27 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:10">
+    <x:row r="4" spans="1:18">
       <x:c r="A4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H4" s="0">
         <x:v>10</x:v>
@@ -701,27 +778,27 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:10">
+    <x:row r="5" spans="1:18">
       <x:c r="A5" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H5" s="0">
         <x:v>-1</x:v>
@@ -733,59 +810,59 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" spans="1:10">
+    <x:row r="6" spans="1:18">
       <x:c r="A6" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>1</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>2</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="J6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:10">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:18">
       <x:c r="A7" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H7" s="0">
         <x:v>1</x:v>
@@ -794,7 +871,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J7" s="0">
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -811,7 +888,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:J3"/>
+  <x:dimension ref="A1:R3"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="17.710625" style="0" customWidth="1"/>
@@ -824,9 +901,17 @@
     <x:col min="8" max="8" width="14.567768" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="11.853482" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="8.282054" style="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14.424911" style="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13.282054" style="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="15" max="15" width="9.853482" style="0" customWidth="1"/>
+    <x:col min="16" max="16" width="13.853482" style="0" customWidth="1"/>
+    <x:col min="17" max="17" width="17.567768" style="0" customWidth="1"/>
+    <x:col min="18" max="18" width="9.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:10">
+    <x:row r="1" spans="1:18">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -857,19 +942,43 @@
       <x:c r="J1" s="1" t="s">
         <x:v>9</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:10">
+      <x:c r="K1" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L1" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="M1" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N1" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="O1" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="P1" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="Q1" s="1" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="R1" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:18">
       <x:c r="A2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>80</x:v>
@@ -881,12 +990,12 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:10">
+    <x:row r="3" spans="1:18">
       <x:c r="A3" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>150</x:v>
@@ -912,7 +1021,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A20"/>
+  <x:dimension ref="A1:A28"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="110.710625" style="0" customWidth="1"/>
@@ -920,102 +1029,142 @@
   <x:sheetData>
     <x:row r="1" spans="1:1">
       <x:c r="A1" s="2" t="s">
-        <x:v>16</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
       <x:c r="A2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1">
       <x:c r="A3" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
       <x:c r="A4" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
       <x:c r="A5" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
       <x:c r="A7" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:1">
       <x:c r="A8" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:1">
       <x:c r="A9" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:1">
       <x:c r="A10" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:1">
       <x:c r="A11" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:1">
       <x:c r="A12" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:1">
       <x:c r="A13" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:1">
       <x:c r="A14" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:1">
       <x:c r="A15" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:1">
       <x:c r="A16" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:1">
       <x:c r="A17" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:1">
       <x:c r="A18" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:1">
       <x:c r="A19" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:1">
       <x:c r="A20" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>43</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:1">
+      <x:c r="A21" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:1">
+      <x:c r="A22" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:1">
+      <x:c r="A23" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:1">
+      <x:c r="A24" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:1">
+      <x:c r="A25" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:1">
+      <x:c r="A26" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" spans="1:1">
+      <x:c r="A27" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:1">
+      <x:c r="A28" s="0" t="s">
+        <x:v>49</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1044,33 +1193,33 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="2" t="s">
-        <x:v>34</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>35</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>36</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
-        <x:v>37</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
       <x:c r="A2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>18</x:v>

</xml_diff>